<commit_message>
feat(verilog): column-aligned port/parameter declarations
Pre-compute alignment widths in Python and format lines before
passing to Jinja2 template. Columns: direction(7), signed(7),
type(5), width(max-width), name. Parameters: '=' aligned to
longest name. All left-aligned with spaces (no tabs).

Comma logic handles cross-group presence (input→output→inout).
</commit_message>
<xml_diff>
--- a/examples/sample_module_sram_wrap.xlsx
+++ b/examples/sample_module_sram_wrap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitLab\AI_Project\excel2design\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00B9DC0-BCAC-4E1C-9277-D2C3707FAEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FDD272-6D58-4511-BE63-AB96FE033BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1837,7 +1837,7 @@
         <v>103</v>
       </c>
       <c r="H52" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" s="3">
         <v>0</v>
@@ -1863,7 +1863,7 @@
         <v>103</v>
       </c>
       <c r="H53" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" s="3">
         <v>0</v>

</xml_diff>